<commit_message>
Fix formula-text conflict in 02_Amortization_Schedule.xlsx: prefix display strings starting with = to prevent openpyxl from treating them as Excel formulas
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-11/02_Amortization_Schedule.xlsx
+++ b/rFLA300/chapter-11/02_Amortization_Schedule.xlsx
@@ -2617,9 +2617,10 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="27">
-        <f>IPMT(rate, per, nper, pv, [fv], [type])</f>
-        <v/>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =IPMT(rate, per, nper, pv, [fv], [type])</t>
+        </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -2628,9 +2629,10 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="27">
-        <f>PPMT(rate, per, nper, pv, [fv], [type])</f>
-        <v/>
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> =PPMT(rate, per, nper, pv, [fv], [type])</t>
+        </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>

</xml_diff>